<commit_message>
Identidad Grupo Canville completa; libro de control operativo semanal, reporte semanal, plan de 30 días y modelo operativo; presentación comercial (PDF/HTML), infografías, mensajes y guion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/ejemplos/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos_EJEMPLO.xlsx
+++ b/ejemplos/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos_EJEMPLO.xlsx
@@ -56,7 +56,7 @@
     <font>
       <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="001B6B73"/>
+      <color rgb="000E7C8B"/>
     </font>
     <font>
       <name val="Abadi"/>
@@ -81,7 +81,7 @@
     <font>
       <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="001B6B73"/>
+      <color rgb="000E7C8B"/>
       <sz val="9"/>
     </font>
     <font>
@@ -123,7 +123,7 @@
     <font>
       <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="001B6B73"/>
+      <color rgb="000E7C8B"/>
       <sz val="12"/>
     </font>
     <font>
@@ -146,7 +146,7 @@
     <font>
       <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="001B6B73"/>
+      <color rgb="000E7C8B"/>
       <sz val="11"/>
     </font>
     <font>
@@ -174,7 +174,7 @@
     <font>
       <name val="Abadi"/>
       <b val="1"/>
-      <color rgb="001B6B73"/>
+      <color rgb="000E7C8B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -799,11 +799,11 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="1B6B73"/>
+              <a:srgbClr val="0E7C8B"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
-                <a:srgbClr val="1B6B73"/>
+                <a:srgbClr val="0E7C8B"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -919,11 +919,11 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="1B6B73"/>
+              <a:srgbClr val="0E7C8B"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
-                <a:srgbClr val="1B6B73"/>
+                <a:srgbClr val="0E7C8B"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -7842,7 +7842,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001B6B73"/>
+    <tabColor rgb="000E7C8B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -9362,7 +9362,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001B6B73"/>
+    <tabColor rgb="000E7C8B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
Productos sin marca ni logotipo: etiqueta genérica en portadas, portada Excel, presentación e infografías; marca opcional y configurable
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/ejemplos/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos_EJEMPLO.xlsx
+++ b/ejemplos/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos_EJEMPLO.xlsx
@@ -1371,7 +1371,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>GRUPO CANVILLE</t>
+          <t>FORMATOS ADMINISTRATIVOS</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -1849,7 +1849,7 @@
       <c r="A41" s="1" t="n"/>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>GRUPO CANVILLE  ·  Formatos administrativos  ·  Para uso interno de tu empresa</t>
+          <t>Formatos administrativos  ·  Para uso interno de tu empresa</t>
         </is>
       </c>
       <c r="G41" s="1" t="n"/>

</xml_diff>